<commit_message>
Initial code for paper
</commit_message>
<xml_diff>
--- a/results/dn/STM_m20_n_1to5by0.2_deg5_c10_rho0.5_rp5_d343_lam0.1_Mxi2000.xlsx
+++ b/results/dn/STM_m20_n_1to5by0.2_deg5_c10_rho0.5_rp5_d343_lam0.1_Mxi2000.xlsx
@@ -48242,6 +48242,366 @@
       <c r="AO100" t="n">
         <v>-0.016337282428717</v>
       </c>
+      <c r="AP100" t="n">
+        <v>-0.105999958470186</v>
+      </c>
+      <c r="AQ100" t="n">
+        <v>-0.0679661329821624</v>
+      </c>
+      <c r="AR100" t="n">
+        <v>0.00514430293055266</v>
+      </c>
+      <c r="AS100" t="n">
+        <v>0.0456577871874654</v>
+      </c>
+      <c r="AT100" t="n">
+        <v>0.0364709939203495</v>
+      </c>
+      <c r="AU100" t="n">
+        <v>0.0152868045840652</v>
+      </c>
+      <c r="AV100" t="n">
+        <v>-0.0325859981454966</v>
+      </c>
+      <c r="AW100" t="n">
+        <v>-0.107206230788768</v>
+      </c>
+      <c r="AX100" t="n">
+        <v>0.0313875331038416</v>
+      </c>
+      <c r="AY100" t="n">
+        <v>0.0107680455915348</v>
+      </c>
+      <c r="AZ100" t="n">
+        <v>-0.00897264464396332</v>
+      </c>
+      <c r="BA100" t="n">
+        <v>-0.0165319665095981</v>
+      </c>
+      <c r="BB100" t="n">
+        <v>-0.0322665921134472</v>
+      </c>
+      <c r="BC100" t="n">
+        <v>-0.0480692709317428</v>
+      </c>
+      <c r="BD100" t="n">
+        <v>-0.063869115202242</v>
+      </c>
+      <c r="BE100" t="n">
+        <v>0.184814606691316</v>
+      </c>
+      <c r="BF100" t="n">
+        <v>0.0135473038051096</v>
+      </c>
+      <c r="BG100" t="n">
+        <v>-0.101039101418792</v>
+      </c>
+      <c r="BH100" t="n">
+        <v>-0.104743248350823</v>
+      </c>
+      <c r="BI100" t="n">
+        <v>-0.106588557522046</v>
+      </c>
+      <c r="BJ100" t="n">
+        <v>-0.0638830664803188</v>
+      </c>
+      <c r="BK100" t="n">
+        <v>0.0235600073059877</v>
+      </c>
+      <c r="BL100" t="n">
+        <v>-0.0478079732742329</v>
+      </c>
+      <c r="BM100" t="n">
+        <v>-0.0228247141749373</v>
+      </c>
+      <c r="BN100" t="n">
+        <v>-0.00263759840213383</v>
+      </c>
+      <c r="BO100" t="n">
+        <v>-0.00346676020955269</v>
+      </c>
+      <c r="BP100" t="n">
+        <v>0.00553917048971234</v>
+      </c>
+      <c r="BQ100" t="n">
+        <v>0.0113659166420016</v>
+      </c>
+      <c r="BR100" t="n">
+        <v>0.0134153371500161</v>
+      </c>
+      <c r="BS100" t="n">
+        <v>-0.0230477854328511</v>
+      </c>
+      <c r="BT100" t="n">
+        <v>-0.0167448810384792</v>
+      </c>
+      <c r="BU100" t="n">
+        <v>-0.0102604253676079</v>
+      </c>
+      <c r="BV100" t="n">
+        <v>-0.0119521764778214</v>
+      </c>
+      <c r="BW100" t="n">
+        <v>-0.0062380518548665</v>
+      </c>
+      <c r="BX100" t="n">
+        <v>0.0000300584385514807</v>
+      </c>
+      <c r="BY100" t="n">
+        <v>0.00638625283657475</v>
+      </c>
+      <c r="BZ100" t="n">
+        <v>-0.00273205329153914</v>
+      </c>
+      <c r="CA100" t="n">
+        <v>-0.0102130982174715</v>
+      </c>
+      <c r="CB100" t="n">
+        <v>-0.0144198118158115</v>
+      </c>
+      <c r="CC100" t="n">
+        <v>-0.0170417268883501</v>
+      </c>
+      <c r="CD100" t="n">
+        <v>-0.0152344123813784</v>
+      </c>
+      <c r="CE100" t="n">
+        <v>-0.0106721989669744</v>
+      </c>
+      <c r="CF100" t="n">
+        <v>-0.00366648105664125</v>
+      </c>
+      <c r="CG100" t="n">
+        <v>-0.00347293159919433</v>
+      </c>
+      <c r="CH100" t="n">
+        <v>-0.0118984537978161</v>
+      </c>
+      <c r="CI100" t="n">
+        <v>-0.0171279036342037</v>
+      </c>
+      <c r="CJ100" t="n">
+        <v>-0.0210723559741773</v>
+      </c>
+      <c r="CK100" t="n">
+        <v>-0.020341145245519</v>
+      </c>
+      <c r="CL100" t="n">
+        <v>-0.0169338629674322</v>
+      </c>
+      <c r="CM100" t="n">
+        <v>-0.0112470942085088</v>
+      </c>
+      <c r="CN100" t="n">
+        <v>0.00582135658832952</v>
+      </c>
+      <c r="CO100" t="n">
+        <v>-0.00604804869981282</v>
+      </c>
+      <c r="CP100" t="n">
+        <v>-0.0153012978195772</v>
+      </c>
+      <c r="CQ100" t="n">
+        <v>-0.0203350127237646</v>
+      </c>
+      <c r="CR100" t="n">
+        <v>-0.0240797364166209</v>
+      </c>
+      <c r="CS100" t="n">
+        <v>-0.0258535589326018</v>
+      </c>
+      <c r="CT100" t="n">
+        <v>-0.0259334356413971</v>
+      </c>
+      <c r="CU100" t="n">
+        <v>0.0113867171404924</v>
+      </c>
+      <c r="CV100" t="n">
+        <v>-0.0000256285632340379</v>
+      </c>
+      <c r="CW100" t="n">
+        <v>-0.01086892175285</v>
+      </c>
+      <c r="CX100" t="n">
+        <v>-0.0170447623543247</v>
+      </c>
+      <c r="CY100" t="n">
+        <v>-0.0256689302480678</v>
+      </c>
+      <c r="CZ100" t="n">
+        <v>-0.0342045951508378</v>
+      </c>
+      <c r="DA100" t="n">
+        <v>-0.0428108888384633</v>
+      </c>
+      <c r="DB100" t="n">
+        <v>0.0139006071066637</v>
+      </c>
+      <c r="DC100" t="n">
+        <v>0.00657976178718516</v>
+      </c>
+      <c r="DD100" t="n">
+        <v>-0.0037143099330434</v>
+      </c>
+      <c r="DE100" t="n">
+        <v>-0.0111531531087371</v>
+      </c>
+      <c r="DF100" t="n">
+        <v>-0.0253634201326367</v>
+      </c>
+      <c r="DG100" t="n">
+        <v>-0.0425885461939076</v>
+      </c>
+      <c r="DH100" t="n">
+        <v>-0.0628406490777315</v>
+      </c>
+      <c r="DI100" t="n">
+        <v>-0.123571037728762</v>
+      </c>
+      <c r="DJ100" t="n">
+        <v>-0.00294532695817352</v>
+      </c>
+      <c r="DK100" t="n">
+        <v>0.0707341652750297</v>
+      </c>
+      <c r="DL100" t="n">
+        <v>0.0634549519364231</v>
+      </c>
+      <c r="DM100" t="n">
+        <v>0.046344589821701</v>
+      </c>
+      <c r="DN100" t="n">
+        <v>-0.00851748654849184</v>
+      </c>
+      <c r="DO100" t="n">
+        <v>-0.101339109162831</v>
+      </c>
+      <c r="DP100" t="n">
+        <v>-0.00300483790567401</v>
+      </c>
+      <c r="DQ100" t="n">
+        <v>-0.0100688079399932</v>
+      </c>
+      <c r="DR100" t="n">
+        <v>-0.0140363032785307</v>
+      </c>
+      <c r="DS100" t="n">
+        <v>-0.0166587205447638</v>
+      </c>
+      <c r="DT100" t="n">
+        <v>-0.0149714429020513</v>
+      </c>
+      <c r="DU100" t="n">
+        <v>-0.0106682013779227</v>
+      </c>
+      <c r="DV100" t="n">
+        <v>-0.0040728421919208</v>
+      </c>
+      <c r="DW100" t="n">
+        <v>0.0706740292148516</v>
+      </c>
+      <c r="DX100" t="n">
+        <v>-0.0139319460476585</v>
+      </c>
+      <c r="DY100" t="n">
+        <v>-0.0651812422198551</v>
+      </c>
+      <c r="DZ100" t="n">
+        <v>-0.065004202327992</v>
+      </c>
+      <c r="EA100" t="n">
+        <v>-0.0521833850664866</v>
+      </c>
+      <c r="EB100" t="n">
+        <v>-0.0123333983882896</v>
+      </c>
+      <c r="EC100" t="n">
+        <v>0.0541624678240314</v>
+      </c>
+      <c r="ED100" t="n">
+        <v>0.0638059569836822</v>
+      </c>
+      <c r="EE100" t="n">
+        <v>-0.0166161631500873</v>
+      </c>
+      <c r="EF100" t="n">
+        <v>-0.0653983325848697</v>
+      </c>
+      <c r="EG100" t="n">
+        <v>-0.0665434408954858</v>
+      </c>
+      <c r="EH100" t="n">
+        <v>-0.0545941456714314</v>
+      </c>
+      <c r="EI100" t="n">
+        <v>-0.0169766950692452</v>
+      </c>
+      <c r="EJ100" t="n">
+        <v>0.0458183556914049</v>
+      </c>
+      <c r="EK100" t="n">
+        <v>0.0457251720066406</v>
+      </c>
+      <c r="EL100" t="n">
+        <v>-0.0149038763345857</v>
+      </c>
+      <c r="EM100" t="n">
+        <v>-0.0519240564223409</v>
+      </c>
+      <c r="EN100" t="n">
+        <v>-0.0540767323532047</v>
+      </c>
+      <c r="EO100" t="n">
+        <v>-0.0457899529858335</v>
+      </c>
+      <c r="EP100" t="n">
+        <v>-0.0183558644630337</v>
+      </c>
+      <c r="EQ100" t="n">
+        <v>0.027751298444847</v>
+      </c>
+      <c r="ER100" t="n">
+        <v>-0.0088365615467901</v>
+      </c>
+      <c r="ES100" t="n">
+        <v>-0.0107456744996076</v>
+      </c>
+      <c r="ET100" t="n">
+        <v>-0.012423548384556</v>
+      </c>
+      <c r="EU100" t="n">
+        <v>-0.0170458534395367</v>
+      </c>
+      <c r="EV100" t="n">
+        <v>-0.0183580069042594</v>
+      </c>
+      <c r="EW100" t="n">
+        <v>-0.0194370181359543</v>
+      </c>
+      <c r="EX100" t="n">
+        <v>-0.0206706655844961</v>
+      </c>
+      <c r="EY100" t="n">
+        <v>-0.10077331911299</v>
+      </c>
+      <c r="EZ100" t="n">
+        <v>-0.0040318396848199</v>
+      </c>
+      <c r="FA100" t="n">
+        <v>0.0538170940684659</v>
+      </c>
+      <c r="FB100" t="n">
+        <v>0.0452055274102241</v>
+      </c>
+      <c r="FC100" t="n">
+        <v>0.0281605824049469</v>
+      </c>
+      <c r="FD100" t="n">
+        <v>-0.0202797384902911</v>
+      </c>
+      <c r="FE100" t="n">
+        <v>-0.100383597796463</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -48367,6 +48727,366 @@
       <c r="AO101" t="n">
         <v>-0.0160040120355426</v>
       </c>
+      <c r="AP101" t="n">
+        <v>-0.106551846678342</v>
+      </c>
+      <c r="AQ101" t="n">
+        <v>-0.0689062222685067</v>
+      </c>
+      <c r="AR101" t="n">
+        <v>0.00599618064691515</v>
+      </c>
+      <c r="AS101" t="n">
+        <v>0.0462253004105565</v>
+      </c>
+      <c r="AT101" t="n">
+        <v>0.0377941378646604</v>
+      </c>
+      <c r="AU101" t="n">
+        <v>0.0156585497276504</v>
+      </c>
+      <c r="AV101" t="n">
+        <v>-0.0319925867441001</v>
+      </c>
+      <c r="AW101" t="n">
+        <v>-0.107390048677004</v>
+      </c>
+      <c r="AX101" t="n">
+        <v>0.0322207092847197</v>
+      </c>
+      <c r="AY101" t="n">
+        <v>0.0116118045332823</v>
+      </c>
+      <c r="AZ101" t="n">
+        <v>-0.00934145473923414</v>
+      </c>
+      <c r="BA101" t="n">
+        <v>-0.0169439271023599</v>
+      </c>
+      <c r="BB101" t="n">
+        <v>-0.0332891330423497</v>
+      </c>
+      <c r="BC101" t="n">
+        <v>-0.0489093858855883</v>
+      </c>
+      <c r="BD101" t="n">
+        <v>-0.0642451959188374</v>
+      </c>
+      <c r="BE101" t="n">
+        <v>0.184465050118866</v>
+      </c>
+      <c r="BF101" t="n">
+        <v>0.013251134731493</v>
+      </c>
+      <c r="BG101" t="n">
+        <v>-0.101595758729954</v>
+      </c>
+      <c r="BH101" t="n">
+        <v>-0.106609796176156</v>
+      </c>
+      <c r="BI101" t="n">
+        <v>-0.107914203781092</v>
+      </c>
+      <c r="BJ101" t="n">
+        <v>-0.0653222649369451</v>
+      </c>
+      <c r="BK101" t="n">
+        <v>0.0236108515271809</v>
+      </c>
+      <c r="BL101" t="n">
+        <v>-0.047437789346576</v>
+      </c>
+      <c r="BM101" t="n">
+        <v>-0.0227168158555577</v>
+      </c>
+      <c r="BN101" t="n">
+        <v>-0.00229480823720233</v>
+      </c>
+      <c r="BO101" t="n">
+        <v>-0.00325785572092198</v>
+      </c>
+      <c r="BP101" t="n">
+        <v>0.00584411611249816</v>
+      </c>
+      <c r="BQ101" t="n">
+        <v>0.0116333222704315</v>
+      </c>
+      <c r="BR101" t="n">
+        <v>0.0132991123482681</v>
+      </c>
+      <c r="BS101" t="n">
+        <v>-0.0225122199862335</v>
+      </c>
+      <c r="BT101" t="n">
+        <v>-0.0162516049419403</v>
+      </c>
+      <c r="BU101" t="n">
+        <v>-0.00963497533287661</v>
+      </c>
+      <c r="BV101" t="n">
+        <v>-0.0114432215623604</v>
+      </c>
+      <c r="BW101" t="n">
+        <v>-0.00573686777976826</v>
+      </c>
+      <c r="BX101" t="n">
+        <v>0.000370219638611152</v>
+      </c>
+      <c r="BY101" t="n">
+        <v>0.00635500496669514</v>
+      </c>
+      <c r="BZ101" t="n">
+        <v>-0.00216478872117848</v>
+      </c>
+      <c r="CA101" t="n">
+        <v>-0.00948858198583488</v>
+      </c>
+      <c r="CB101" t="n">
+        <v>-0.0137068614554867</v>
+      </c>
+      <c r="CC101" t="n">
+        <v>-0.0164514813320467</v>
+      </c>
+      <c r="CD101" t="n">
+        <v>-0.0148155274363574</v>
+      </c>
+      <c r="CE101" t="n">
+        <v>-0.0105170528667989</v>
+      </c>
+      <c r="CF101" t="n">
+        <v>-0.00389194335920703</v>
+      </c>
+      <c r="CG101" t="n">
+        <v>-0.00336894555433298</v>
+      </c>
+      <c r="CH101" t="n">
+        <v>-0.0114849528556198</v>
+      </c>
+      <c r="CI101" t="n">
+        <v>-0.0166775596993702</v>
+      </c>
+      <c r="CJ101" t="n">
+        <v>-0.0208252146006339</v>
+      </c>
+      <c r="CK101" t="n">
+        <v>-0.0201676561628113</v>
+      </c>
+      <c r="CL101" t="n">
+        <v>-0.0168294200186348</v>
+      </c>
+      <c r="CM101" t="n">
+        <v>-0.0113170251015299</v>
+      </c>
+      <c r="CN101" t="n">
+        <v>0.00576764982234263</v>
+      </c>
+      <c r="CO101" t="n">
+        <v>-0.00553741860328353</v>
+      </c>
+      <c r="CP101" t="n">
+        <v>-0.0147803064184425</v>
+      </c>
+      <c r="CQ101" t="n">
+        <v>-0.0198343151839644</v>
+      </c>
+      <c r="CR101" t="n">
+        <v>-0.0235743107381373</v>
+      </c>
+      <c r="CS101" t="n">
+        <v>-0.0251476852052021</v>
+      </c>
+      <c r="CT101" t="n">
+        <v>-0.0250530395167479</v>
+      </c>
+      <c r="CU101" t="n">
+        <v>0.0112579754767958</v>
+      </c>
+      <c r="CV101" t="n">
+        <v>0.000452953509642056</v>
+      </c>
+      <c r="CW101" t="n">
+        <v>-0.0106577652470102</v>
+      </c>
+      <c r="CX101" t="n">
+        <v>-0.0168182246866733</v>
+      </c>
+      <c r="CY101" t="n">
+        <v>-0.0255984826992894</v>
+      </c>
+      <c r="CZ101" t="n">
+        <v>-0.0338665404498724</v>
+      </c>
+      <c r="DA101" t="n">
+        <v>-0.0421805735280629</v>
+      </c>
+      <c r="DB101" t="n">
+        <v>0.0128450343554632</v>
+      </c>
+      <c r="DC101" t="n">
+        <v>0.00646314253037392</v>
+      </c>
+      <c r="DD101" t="n">
+        <v>-0.00406703385666055</v>
+      </c>
+      <c r="DE101" t="n">
+        <v>-0.0113708561511758</v>
+      </c>
+      <c r="DF101" t="n">
+        <v>-0.0255623872906969</v>
+      </c>
+      <c r="DG101" t="n">
+        <v>-0.0420014028217034</v>
+      </c>
+      <c r="DH101" t="n">
+        <v>-0.0614017605850908</v>
+      </c>
+      <c r="DI101" t="n">
+        <v>-0.123741437289412</v>
+      </c>
+      <c r="DJ101" t="n">
+        <v>-0.00225550432359191</v>
+      </c>
+      <c r="DK101" t="n">
+        <v>0.0708924877592342</v>
+      </c>
+      <c r="DL101" t="n">
+        <v>0.0646449896504886</v>
+      </c>
+      <c r="DM101" t="n">
+        <v>0.0466866069552893</v>
+      </c>
+      <c r="DN101" t="n">
+        <v>-0.00757988259451431</v>
+      </c>
+      <c r="DO101" t="n">
+        <v>-0.101011569424602</v>
+      </c>
+      <c r="DP101" t="n">
+        <v>-0.00282860231082577</v>
+      </c>
+      <c r="DQ101" t="n">
+        <v>-0.00962192430917374</v>
+      </c>
+      <c r="DR101" t="n">
+        <v>-0.0134733299396778</v>
+      </c>
+      <c r="DS101" t="n">
+        <v>-0.0162224862984408</v>
+      </c>
+      <c r="DT101" t="n">
+        <v>-0.0145641362005007</v>
+      </c>
+      <c r="DU101" t="n">
+        <v>-0.0103707609119014</v>
+      </c>
+      <c r="DV101" t="n">
+        <v>-0.00398861415812052</v>
+      </c>
+      <c r="DW101" t="n">
+        <v>0.0702770231637627</v>
+      </c>
+      <c r="DX101" t="n">
+        <v>-0.0137028138948497</v>
+      </c>
+      <c r="DY101" t="n">
+        <v>-0.0640158536026531</v>
+      </c>
+      <c r="DZ101" t="n">
+        <v>-0.0647236022476319</v>
+      </c>
+      <c r="EA101" t="n">
+        <v>-0.0515499520524509</v>
+      </c>
+      <c r="EB101" t="n">
+        <v>-0.0125563055016214</v>
+      </c>
+      <c r="EC101" t="n">
+        <v>0.0534198999250598</v>
+      </c>
+      <c r="ED101" t="n">
+        <v>0.0639430811937126</v>
+      </c>
+      <c r="EE101" t="n">
+        <v>-0.0166437148197014</v>
+      </c>
+      <c r="EF101" t="n">
+        <v>-0.0650406996938989</v>
+      </c>
+      <c r="EG101" t="n">
+        <v>-0.0671348071729243</v>
+      </c>
+      <c r="EH101" t="n">
+        <v>-0.0547225678111294</v>
+      </c>
+      <c r="EI101" t="n">
+        <v>-0.0174757735747919</v>
+      </c>
+      <c r="EJ101" t="n">
+        <v>0.0455020666221556</v>
+      </c>
+      <c r="EK101" t="n">
+        <v>0.04632063372836</v>
+      </c>
+      <c r="EL101" t="n">
+        <v>-0.0147003918016228</v>
+      </c>
+      <c r="EM101" t="n">
+        <v>-0.0516639501650685</v>
+      </c>
+      <c r="EN101" t="n">
+        <v>-0.0544602118004679</v>
+      </c>
+      <c r="EO101" t="n">
+        <v>-0.0457439035565524</v>
+      </c>
+      <c r="EP101" t="n">
+        <v>-0.0183335682491298</v>
+      </c>
+      <c r="EQ101" t="n">
+        <v>0.0282862662949971</v>
+      </c>
+      <c r="ER101" t="n">
+        <v>-0.00915351857122843</v>
+      </c>
+      <c r="ES101" t="n">
+        <v>-0.0104979453181972</v>
+      </c>
+      <c r="ET101" t="n">
+        <v>-0.0120586049894</v>
+      </c>
+      <c r="EU101" t="n">
+        <v>-0.0168268194640229</v>
+      </c>
+      <c r="EV101" t="n">
+        <v>-0.0181981997201163</v>
+      </c>
+      <c r="EW101" t="n">
+        <v>-0.0192235587638313</v>
+      </c>
+      <c r="EX101" t="n">
+        <v>-0.0205851616689031</v>
+      </c>
+      <c r="EY101" t="n">
+        <v>-0.101251990549701</v>
+      </c>
+      <c r="EZ101" t="n">
+        <v>-0.00380994696008678</v>
+      </c>
+      <c r="FA101" t="n">
+        <v>0.053414261935146</v>
+      </c>
+      <c r="FB101" t="n">
+        <v>0.0455614557011862</v>
+      </c>
+      <c r="FC101" t="n">
+        <v>0.0279198275661188</v>
+      </c>
+      <c r="FD101" t="n">
+        <v>-0.0196203742539297</v>
+      </c>
+      <c r="FE101" t="n">
+        <v>-0.099713537097665</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -48492,6 +49212,366 @@
       <c r="AO102" t="n">
         <v>-0.0165473423308738</v>
       </c>
+      <c r="AP102" t="n">
+        <v>-0.106419652353299</v>
+      </c>
+      <c r="AQ102" t="n">
+        <v>-0.0688348080434882</v>
+      </c>
+      <c r="AR102" t="n">
+        <v>0.00560228322356434</v>
+      </c>
+      <c r="AS102" t="n">
+        <v>0.0458442696180946</v>
+      </c>
+      <c r="AT102" t="n">
+        <v>0.0369612783483048</v>
+      </c>
+      <c r="AU102" t="n">
+        <v>0.0155728953423449</v>
+      </c>
+      <c r="AV102" t="n">
+        <v>-0.0323102601903038</v>
+      </c>
+      <c r="AW102" t="n">
+        <v>-0.106850008607501</v>
+      </c>
+      <c r="AX102" t="n">
+        <v>0.0316994876704898</v>
+      </c>
+      <c r="AY102" t="n">
+        <v>0.0115390755346423</v>
+      </c>
+      <c r="AZ102" t="n">
+        <v>-0.00845737826673714</v>
+      </c>
+      <c r="BA102" t="n">
+        <v>-0.0163090672293264</v>
+      </c>
+      <c r="BB102" t="n">
+        <v>-0.0323944038670945</v>
+      </c>
+      <c r="BC102" t="n">
+        <v>-0.0484975424267089</v>
+      </c>
+      <c r="BD102" t="n">
+        <v>-0.0645861896197863</v>
+      </c>
+      <c r="BE102" t="n">
+        <v>0.185700472715047</v>
+      </c>
+      <c r="BF102" t="n">
+        <v>0.0140074891916961</v>
+      </c>
+      <c r="BG102" t="n">
+        <v>-0.100049111811756</v>
+      </c>
+      <c r="BH102" t="n">
+        <v>-0.104925648011706</v>
+      </c>
+      <c r="BI102" t="n">
+        <v>-0.106867421759685</v>
+      </c>
+      <c r="BJ102" t="n">
+        <v>-0.0645955662701379</v>
+      </c>
+      <c r="BK102" t="n">
+        <v>0.0222945214557707</v>
+      </c>
+      <c r="BL102" t="n">
+        <v>-0.0469987806728653</v>
+      </c>
+      <c r="BM102" t="n">
+        <v>-0.0231112597727253</v>
+      </c>
+      <c r="BN102" t="n">
+        <v>-0.00313904865505317</v>
+      </c>
+      <c r="BO102" t="n">
+        <v>-0.00397470321140887</v>
+      </c>
+      <c r="BP102" t="n">
+        <v>0.0052010781699652</v>
+      </c>
+      <c r="BQ102" t="n">
+        <v>0.0111113262793775</v>
+      </c>
+      <c r="BR102" t="n">
+        <v>0.013748214652504</v>
+      </c>
+      <c r="BS102" t="n">
+        <v>-0.0227939129943786</v>
+      </c>
+      <c r="BT102" t="n">
+        <v>-0.0166241210495475</v>
+      </c>
+      <c r="BU102" t="n">
+        <v>-0.00981684421449578</v>
+      </c>
+      <c r="BV102" t="n">
+        <v>-0.0115059702968174</v>
+      </c>
+      <c r="BW102" t="n">
+        <v>-0.00569340332216465</v>
+      </c>
+      <c r="BX102" t="n">
+        <v>0.000385831046293195</v>
+      </c>
+      <c r="BY102" t="n">
+        <v>0.00675664697309921</v>
+      </c>
+      <c r="BZ102" t="n">
+        <v>-0.00274793149088817</v>
+      </c>
+      <c r="CA102" t="n">
+        <v>-0.00985826805740325</v>
+      </c>
+      <c r="CB102" t="n">
+        <v>-0.0135950287006758</v>
+      </c>
+      <c r="CC102" t="n">
+        <v>-0.0163097592902092</v>
+      </c>
+      <c r="CD102" t="n">
+        <v>-0.0145786276220865</v>
+      </c>
+      <c r="CE102" t="n">
+        <v>-0.0104496245126473</v>
+      </c>
+      <c r="CF102" t="n">
+        <v>-0.00387547101496672</v>
+      </c>
+      <c r="CG102" t="n">
+        <v>-0.00358471163849488</v>
+      </c>
+      <c r="CH102" t="n">
+        <v>-0.0116828507375646</v>
+      </c>
+      <c r="CI102" t="n">
+        <v>-0.0164360336729996</v>
+      </c>
+      <c r="CJ102" t="n">
+        <v>-0.0205619769266148</v>
+      </c>
+      <c r="CK102" t="n">
+        <v>-0.0198687184607458</v>
+      </c>
+      <c r="CL102" t="n">
+        <v>-0.0168661184972883</v>
+      </c>
+      <c r="CM102" t="n">
+        <v>-0.0114968615627337</v>
+      </c>
+      <c r="CN102" t="n">
+        <v>0.00565624317787787</v>
+      </c>
+      <c r="CO102" t="n">
+        <v>-0.00568733181565649</v>
+      </c>
+      <c r="CP102" t="n">
+        <v>-0.0144697694659</v>
+      </c>
+      <c r="CQ102" t="n">
+        <v>-0.0195747297801513</v>
+      </c>
+      <c r="CR102" t="n">
+        <v>-0.0232329977797352</v>
+      </c>
+      <c r="CS102" t="n">
+        <v>-0.0251590224454134</v>
+      </c>
+      <c r="CT102" t="n">
+        <v>-0.0252907164887019</v>
+      </c>
+      <c r="CU102" t="n">
+        <v>0.0115763348237153</v>
+      </c>
+      <c r="CV102" t="n">
+        <v>0.000393251826322715</v>
+      </c>
+      <c r="CW102" t="n">
+        <v>-0.010407708989371</v>
+      </c>
+      <c r="CX102" t="n">
+        <v>-0.0166843403812744</v>
+      </c>
+      <c r="CY102" t="n">
+        <v>-0.0252597345685077</v>
+      </c>
+      <c r="CZ102" t="n">
+        <v>-0.0337485480508012</v>
+      </c>
+      <c r="DA102" t="n">
+        <v>-0.0421100835429479</v>
+      </c>
+      <c r="DB102" t="n">
+        <v>0.0141188776392169</v>
+      </c>
+      <c r="DC102" t="n">
+        <v>0.00669315025883045</v>
+      </c>
+      <c r="DD102" t="n">
+        <v>-0.0039766506122322</v>
+      </c>
+      <c r="DE102" t="n">
+        <v>-0.0115146173766855</v>
+      </c>
+      <c r="DF102" t="n">
+        <v>-0.0255250489029582</v>
+      </c>
+      <c r="DG102" t="n">
+        <v>-0.0422082893687987</v>
+      </c>
+      <c r="DH102" t="n">
+        <v>-0.0615469176331602</v>
+      </c>
+      <c r="DI102" t="n">
+        <v>-0.125073753527841</v>
+      </c>
+      <c r="DJ102" t="n">
+        <v>-0.00281846156651318</v>
+      </c>
+      <c r="DK102" t="n">
+        <v>0.0706697185307161</v>
+      </c>
+      <c r="DL102" t="n">
+        <v>0.0638438996607062</v>
+      </c>
+      <c r="DM102" t="n">
+        <v>0.0464046509585886</v>
+      </c>
+      <c r="DN102" t="n">
+        <v>-0.00873126597490501</v>
+      </c>
+      <c r="DO102" t="n">
+        <v>-0.101829858507855</v>
+      </c>
+      <c r="DP102" t="n">
+        <v>-0.00257351295421659</v>
+      </c>
+      <c r="DQ102" t="n">
+        <v>-0.00987599385726995</v>
+      </c>
+      <c r="DR102" t="n">
+        <v>-0.0137280173302651</v>
+      </c>
+      <c r="DS102" t="n">
+        <v>-0.0164486228576422</v>
+      </c>
+      <c r="DT102" t="n">
+        <v>-0.0146993879800004</v>
+      </c>
+      <c r="DU102" t="n">
+        <v>-0.0104942663446834</v>
+      </c>
+      <c r="DV102" t="n">
+        <v>-0.00378329601694907</v>
+      </c>
+      <c r="DW102" t="n">
+        <v>0.0720220183848064</v>
+      </c>
+      <c r="DX102" t="n">
+        <v>-0.0138959947868372</v>
+      </c>
+      <c r="DY102" t="n">
+        <v>-0.0648090153979164</v>
+      </c>
+      <c r="DZ102" t="n">
+        <v>-0.0651460148631835</v>
+      </c>
+      <c r="EA102" t="n">
+        <v>-0.0520536489700978</v>
+      </c>
+      <c r="EB102" t="n">
+        <v>-0.0122438371590861</v>
+      </c>
+      <c r="EC102" t="n">
+        <v>0.0545313308152153</v>
+      </c>
+      <c r="ED102" t="n">
+        <v>0.0653985475704214</v>
+      </c>
+      <c r="EE102" t="n">
+        <v>-0.0167592469465874</v>
+      </c>
+      <c r="EF102" t="n">
+        <v>-0.0654463889574017</v>
+      </c>
+      <c r="EG102" t="n">
+        <v>-0.0671711906245445</v>
+      </c>
+      <c r="EH102" t="n">
+        <v>-0.0548848634364901</v>
+      </c>
+      <c r="EI102" t="n">
+        <v>-0.0171373619047042</v>
+      </c>
+      <c r="EJ102" t="n">
+        <v>0.0463141961224283</v>
+      </c>
+      <c r="EK102" t="n">
+        <v>0.0470673321316445</v>
+      </c>
+      <c r="EL102" t="n">
+        <v>-0.014753864965527</v>
+      </c>
+      <c r="EM102" t="n">
+        <v>-0.0516124534003875</v>
+      </c>
+      <c r="EN102" t="n">
+        <v>-0.0541482508434757</v>
+      </c>
+      <c r="EO102" t="n">
+        <v>-0.0455914255795228</v>
+      </c>
+      <c r="EP102" t="n">
+        <v>-0.0181097488596054</v>
+      </c>
+      <c r="EQ102" t="n">
+        <v>0.0284964032185574</v>
+      </c>
+      <c r="ER102" t="n">
+        <v>-0.00834039745450766</v>
+      </c>
+      <c r="ES102" t="n">
+        <v>-0.0105502841687318</v>
+      </c>
+      <c r="ET102" t="n">
+        <v>-0.0122263625584018</v>
+      </c>
+      <c r="EU102" t="n">
+        <v>-0.0169666350171275</v>
+      </c>
+      <c r="EV102" t="n">
+        <v>-0.0181891014863754</v>
+      </c>
+      <c r="EW102" t="n">
+        <v>-0.0192714473027004</v>
+      </c>
+      <c r="EX102" t="n">
+        <v>-0.0201736189078549</v>
+      </c>
+      <c r="EY102" t="n">
+        <v>-0.101741751233424</v>
+      </c>
+      <c r="EZ102" t="n">
+        <v>-0.00386360129365467</v>
+      </c>
+      <c r="FA102" t="n">
+        <v>0.0537029568559135</v>
+      </c>
+      <c r="FB102" t="n">
+        <v>0.0454316786913359</v>
+      </c>
+      <c r="FC102" t="n">
+        <v>0.0281987193013397</v>
+      </c>
+      <c r="FD102" t="n">
+        <v>-0.0202993427747532</v>
+      </c>
+      <c r="FE102" t="n">
+        <v>-0.100266947836502</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -48617,6 +49697,366 @@
       <c r="AO103" t="n">
         <v>-0.0162387729281515</v>
       </c>
+      <c r="AP103" t="n">
+        <v>-0.106112814540158</v>
+      </c>
+      <c r="AQ103" t="n">
+        <v>-0.0693008367418657</v>
+      </c>
+      <c r="AR103" t="n">
+        <v>0.0055126084786144</v>
+      </c>
+      <c r="AS103" t="n">
+        <v>0.0458382870322665</v>
+      </c>
+      <c r="AT103" t="n">
+        <v>0.0373723400242556</v>
+      </c>
+      <c r="AU103" t="n">
+        <v>0.0154539847683685</v>
+      </c>
+      <c r="AV103" t="n">
+        <v>-0.0323489848686962</v>
+      </c>
+      <c r="AW103" t="n">
+        <v>-0.107411155288286</v>
+      </c>
+      <c r="AX103" t="n">
+        <v>0.0309697937816056</v>
+      </c>
+      <c r="AY103" t="n">
+        <v>0.0112122230721002</v>
+      </c>
+      <c r="AZ103" t="n">
+        <v>-0.00835407093163805</v>
+      </c>
+      <c r="BA103" t="n">
+        <v>-0.0162283599114523</v>
+      </c>
+      <c r="BB103" t="n">
+        <v>-0.0322840511174514</v>
+      </c>
+      <c r="BC103" t="n">
+        <v>-0.0484462462581681</v>
+      </c>
+      <c r="BD103" t="n">
+        <v>-0.0645740809490386</v>
+      </c>
+      <c r="BE103" t="n">
+        <v>0.184769606252804</v>
+      </c>
+      <c r="BF103" t="n">
+        <v>0.0132306878444733</v>
+      </c>
+      <c r="BG103" t="n">
+        <v>-0.100218066843116</v>
+      </c>
+      <c r="BH103" t="n">
+        <v>-0.10590967199223</v>
+      </c>
+      <c r="BI103" t="n">
+        <v>-0.106949113185026</v>
+      </c>
+      <c r="BJ103" t="n">
+        <v>-0.0648962825902157</v>
+      </c>
+      <c r="BK103" t="n">
+        <v>0.0228200592063148</v>
+      </c>
+      <c r="BL103" t="n">
+        <v>-0.0476720858788447</v>
+      </c>
+      <c r="BM103" t="n">
+        <v>-0.0229008820396184</v>
+      </c>
+      <c r="BN103" t="n">
+        <v>-0.00300238622156497</v>
+      </c>
+      <c r="BO103" t="n">
+        <v>-0.00348638629561209</v>
+      </c>
+      <c r="BP103" t="n">
+        <v>0.00579273056645704</v>
+      </c>
+      <c r="BQ103" t="n">
+        <v>0.0118617888677663</v>
+      </c>
+      <c r="BR103" t="n">
+        <v>0.0142452835554465</v>
+      </c>
+      <c r="BS103" t="n">
+        <v>-0.0228716704214374</v>
+      </c>
+      <c r="BT103" t="n">
+        <v>-0.0163515731197362</v>
+      </c>
+      <c r="BU103" t="n">
+        <v>-0.00986655656147187</v>
+      </c>
+      <c r="BV103" t="n">
+        <v>-0.0114063663585184</v>
+      </c>
+      <c r="BW103" t="n">
+        <v>-0.00562771906554124</v>
+      </c>
+      <c r="BX103" t="n">
+        <v>0.000430151345314894</v>
+      </c>
+      <c r="BY103" t="n">
+        <v>0.00655923176610505</v>
+      </c>
+      <c r="BZ103" t="n">
+        <v>-0.00252292780875388</v>
+      </c>
+      <c r="CA103" t="n">
+        <v>-0.00950596737041425</v>
+      </c>
+      <c r="CB103" t="n">
+        <v>-0.0135403211311395</v>
+      </c>
+      <c r="CC103" t="n">
+        <v>-0.0161646700020787</v>
+      </c>
+      <c r="CD103" t="n">
+        <v>-0.0144852829288066</v>
+      </c>
+      <c r="CE103" t="n">
+        <v>-0.0104399689032225</v>
+      </c>
+      <c r="CF103" t="n">
+        <v>-0.00402222534825548</v>
+      </c>
+      <c r="CG103" t="n">
+        <v>-0.0034968192682226</v>
+      </c>
+      <c r="CH103" t="n">
+        <v>-0.0113523442027158</v>
+      </c>
+      <c r="CI103" t="n">
+        <v>-0.0164070668414255</v>
+      </c>
+      <c r="CJ103" t="n">
+        <v>-0.0203914217324056</v>
+      </c>
+      <c r="CK103" t="n">
+        <v>-0.0197046291086003</v>
+      </c>
+      <c r="CL103" t="n">
+        <v>-0.0167254756119066</v>
+      </c>
+      <c r="CM103" t="n">
+        <v>-0.0114829720657422</v>
+      </c>
+      <c r="CN103" t="n">
+        <v>0.00581804700637364</v>
+      </c>
+      <c r="CO103" t="n">
+        <v>-0.00547379509918559</v>
+      </c>
+      <c r="CP103" t="n">
+        <v>-0.0145448061463328</v>
+      </c>
+      <c r="CQ103" t="n">
+        <v>-0.0195893744008431</v>
+      </c>
+      <c r="CR103" t="n">
+        <v>-0.0233009124238372</v>
+      </c>
+      <c r="CS103" t="n">
+        <v>-0.0252744579033634</v>
+      </c>
+      <c r="CT103" t="n">
+        <v>-0.0254817034275331</v>
+      </c>
+      <c r="CU103" t="n">
+        <v>0.0117689215699029</v>
+      </c>
+      <c r="CV103" t="n">
+        <v>0.000646810475352739</v>
+      </c>
+      <c r="CW103" t="n">
+        <v>-0.0102837274046305</v>
+      </c>
+      <c r="CX103" t="n">
+        <v>-0.0164539259355038</v>
+      </c>
+      <c r="CY103" t="n">
+        <v>-0.0251055597395832</v>
+      </c>
+      <c r="CZ103" t="n">
+        <v>-0.0336483579083923</v>
+      </c>
+      <c r="DA103" t="n">
+        <v>-0.0420735573955169</v>
+      </c>
+      <c r="DB103" t="n">
+        <v>0.0140897626975867</v>
+      </c>
+      <c r="DC103" t="n">
+        <v>0.00678708036162157</v>
+      </c>
+      <c r="DD103" t="n">
+        <v>-0.00382279759692513</v>
+      </c>
+      <c r="DE103" t="n">
+        <v>-0.0112792574365021</v>
+      </c>
+      <c r="DF103" t="n">
+        <v>-0.0254199557864916</v>
+      </c>
+      <c r="DG103" t="n">
+        <v>-0.0421975890571414</v>
+      </c>
+      <c r="DH103" t="n">
+        <v>-0.061662857088326</v>
+      </c>
+      <c r="DI103" t="n">
+        <v>-0.123407039322379</v>
+      </c>
+      <c r="DJ103" t="n">
+        <v>-0.0027238856530326</v>
+      </c>
+      <c r="DK103" t="n">
+        <v>0.0694081752568556</v>
+      </c>
+      <c r="DL103" t="n">
+        <v>0.0632683428460203</v>
+      </c>
+      <c r="DM103" t="n">
+        <v>0.0453147007133016</v>
+      </c>
+      <c r="DN103" t="n">
+        <v>-0.00886371939232787</v>
+      </c>
+      <c r="DO103" t="n">
+        <v>-0.101314963612544</v>
+      </c>
+      <c r="DP103" t="n">
+        <v>-0.0027052371731759</v>
+      </c>
+      <c r="DQ103" t="n">
+        <v>-0.00985600003874608</v>
+      </c>
+      <c r="DR103" t="n">
+        <v>-0.014014987912468</v>
+      </c>
+      <c r="DS103" t="n">
+        <v>-0.0167794339495245</v>
+      </c>
+      <c r="DT103" t="n">
+        <v>-0.0151119208852138</v>
+      </c>
+      <c r="DU103" t="n">
+        <v>-0.0110387850712427</v>
+      </c>
+      <c r="DV103" t="n">
+        <v>-0.00455169986776662</v>
+      </c>
+      <c r="DW103" t="n">
+        <v>0.0703685386418879</v>
+      </c>
+      <c r="DX103" t="n">
+        <v>-0.0137325492352828</v>
+      </c>
+      <c r="DY103" t="n">
+        <v>-0.0639155395147746</v>
+      </c>
+      <c r="DZ103" t="n">
+        <v>-0.0646724049344547</v>
+      </c>
+      <c r="EA103" t="n">
+        <v>-0.0514575566658492</v>
+      </c>
+      <c r="EB103" t="n">
+        <v>-0.012665559297749</v>
+      </c>
+      <c r="EC103" t="n">
+        <v>0.0529442349192639</v>
+      </c>
+      <c r="ED103" t="n">
+        <v>0.063986227403673</v>
+      </c>
+      <c r="EE103" t="n">
+        <v>-0.0166415647725982</v>
+      </c>
+      <c r="EF103" t="n">
+        <v>-0.0648888926667983</v>
+      </c>
+      <c r="EG103" t="n">
+        <v>-0.0669895669362081</v>
+      </c>
+      <c r="EH103" t="n">
+        <v>-0.0545347300114442</v>
+      </c>
+      <c r="EI103" t="n">
+        <v>-0.0176045874828576</v>
+      </c>
+      <c r="EJ103" t="n">
+        <v>0.0449417593044164</v>
+      </c>
+      <c r="EK103" t="n">
+        <v>0.04627927398715</v>
+      </c>
+      <c r="EL103" t="n">
+        <v>-0.0148341336822218</v>
+      </c>
+      <c r="EM103" t="n">
+        <v>-0.0516985255050607</v>
+      </c>
+      <c r="EN103" t="n">
+        <v>-0.0544975919899179</v>
+      </c>
+      <c r="EO103" t="n">
+        <v>-0.0456947980789393</v>
+      </c>
+      <c r="EP103" t="n">
+        <v>-0.0185314079076881</v>
+      </c>
+      <c r="EQ103" t="n">
+        <v>0.0278322110484872</v>
+      </c>
+      <c r="ER103" t="n">
+        <v>-0.00853977063681825</v>
+      </c>
+      <c r="ES103" t="n">
+        <v>-0.0105676016336358</v>
+      </c>
+      <c r="ET103" t="n">
+        <v>-0.0125231263287126</v>
+      </c>
+      <c r="EU103" t="n">
+        <v>-0.0171253838247697</v>
+      </c>
+      <c r="EV103" t="n">
+        <v>-0.0182677088146588</v>
+      </c>
+      <c r="EW103" t="n">
+        <v>-0.0191768364058045</v>
+      </c>
+      <c r="EX103" t="n">
+        <v>-0.0199804206293112</v>
+      </c>
+      <c r="EY103" t="n">
+        <v>-0.101374419505451</v>
+      </c>
+      <c r="EZ103" t="n">
+        <v>-0.00405211145572222</v>
+      </c>
+      <c r="FA103" t="n">
+        <v>0.0528368203904412</v>
+      </c>
+      <c r="FB103" t="n">
+        <v>0.0452202864095834</v>
+      </c>
+      <c r="FC103" t="n">
+        <v>0.0277288289180324</v>
+      </c>
+      <c r="FD103" t="n">
+        <v>-0.0199053003456531</v>
+      </c>
+      <c r="FE103" t="n">
+        <v>-0.0994109889292742</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -48742,6 +50182,366 @@
       <c r="AO104" t="n">
         <v>-0.0168336412157096</v>
       </c>
+      <c r="AP104" t="n">
+        <v>-0.106253537075398</v>
+      </c>
+      <c r="AQ104" t="n">
+        <v>-0.0689052919354104</v>
+      </c>
+      <c r="AR104" t="n">
+        <v>0.00560165325539473</v>
+      </c>
+      <c r="AS104" t="n">
+        <v>0.046502488940655</v>
+      </c>
+      <c r="AT104" t="n">
+        <v>0.0373108767330717</v>
+      </c>
+      <c r="AU104" t="n">
+        <v>0.0157098029261526</v>
+      </c>
+      <c r="AV104" t="n">
+        <v>-0.0324690532182812</v>
+      </c>
+      <c r="AW104" t="n">
+        <v>-0.107185678082765</v>
+      </c>
+      <c r="AX104" t="n">
+        <v>0.0313843320901636</v>
+      </c>
+      <c r="AY104" t="n">
+        <v>0.0112149148030642</v>
+      </c>
+      <c r="AZ104" t="n">
+        <v>-0.00848601145515422</v>
+      </c>
+      <c r="BA104" t="n">
+        <v>-0.0159954984954886</v>
+      </c>
+      <c r="BB104" t="n">
+        <v>-0.0322105860896586</v>
+      </c>
+      <c r="BC104" t="n">
+        <v>-0.0481346146884581</v>
+      </c>
+      <c r="BD104" t="n">
+        <v>-0.0640099499768766</v>
+      </c>
+      <c r="BE104" t="n">
+        <v>0.184895427897798</v>
+      </c>
+      <c r="BF104" t="n">
+        <v>0.0132716871869885</v>
+      </c>
+      <c r="BG104" t="n">
+        <v>-0.101274036908937</v>
+      </c>
+      <c r="BH104" t="n">
+        <v>-0.104994264907509</v>
+      </c>
+      <c r="BI104" t="n">
+        <v>-0.107211682310561</v>
+      </c>
+      <c r="BJ104" t="n">
+        <v>-0.0643743490281121</v>
+      </c>
+      <c r="BK104" t="n">
+        <v>0.0227566532210913</v>
+      </c>
+      <c r="BL104" t="n">
+        <v>-0.0475817488463671</v>
+      </c>
+      <c r="BM104" t="n">
+        <v>-0.0228023116023666</v>
+      </c>
+      <c r="BN104" t="n">
+        <v>-0.00272735802958019</v>
+      </c>
+      <c r="BO104" t="n">
+        <v>-0.00365248620495256</v>
+      </c>
+      <c r="BP104" t="n">
+        <v>0.00564639415712592</v>
+      </c>
+      <c r="BQ104" t="n">
+        <v>0.0116675504381315</v>
+      </c>
+      <c r="BR104" t="n">
+        <v>0.0140883184421965</v>
+      </c>
+      <c r="BS104" t="n">
+        <v>-0.0229297579298324</v>
+      </c>
+      <c r="BT104" t="n">
+        <v>-0.0163575174400973</v>
+      </c>
+      <c r="BU104" t="n">
+        <v>-0.00974536303109362</v>
+      </c>
+      <c r="BV104" t="n">
+        <v>-0.0114844964693584</v>
+      </c>
+      <c r="BW104" t="n">
+        <v>-0.00575621016326732</v>
+      </c>
+      <c r="BX104" t="n">
+        <v>0.00034179952375745</v>
+      </c>
+      <c r="BY104" t="n">
+        <v>0.00648398439145079</v>
+      </c>
+      <c r="BZ104" t="n">
+        <v>-0.00289036930908738</v>
+      </c>
+      <c r="CA104" t="n">
+        <v>-0.00986497461970181</v>
+      </c>
+      <c r="CB104" t="n">
+        <v>-0.0138465753481095</v>
+      </c>
+      <c r="CC104" t="n">
+        <v>-0.0165556249702146</v>
+      </c>
+      <c r="CD104" t="n">
+        <v>-0.0149655699852444</v>
+      </c>
+      <c r="CE104" t="n">
+        <v>-0.0107626230100629</v>
+      </c>
+      <c r="CF104" t="n">
+        <v>-0.00428025510612296</v>
+      </c>
+      <c r="CG104" t="n">
+        <v>-0.00355885892430975</v>
+      </c>
+      <c r="CH104" t="n">
+        <v>-0.0114597092711849</v>
+      </c>
+      <c r="CI104" t="n">
+        <v>-0.0165077025224857</v>
+      </c>
+      <c r="CJ104" t="n">
+        <v>-0.0205740222085788</v>
+      </c>
+      <c r="CK104" t="n">
+        <v>-0.0201423498456777</v>
+      </c>
+      <c r="CL104" t="n">
+        <v>-0.0171586838393429</v>
+      </c>
+      <c r="CM104" t="n">
+        <v>-0.0120396982460718</v>
+      </c>
+      <c r="CN104" t="n">
+        <v>0.00564860911696927</v>
+      </c>
+      <c r="CO104" t="n">
+        <v>-0.00572246590178929</v>
+      </c>
+      <c r="CP104" t="n">
+        <v>-0.0147741744292309</v>
+      </c>
+      <c r="CQ104" t="n">
+        <v>-0.0198195125053911</v>
+      </c>
+      <c r="CR104" t="n">
+        <v>-0.0237451518479999</v>
+      </c>
+      <c r="CS104" t="n">
+        <v>-0.0256319490784498</v>
+      </c>
+      <c r="CT104" t="n">
+        <v>-0.025862004845034</v>
+      </c>
+      <c r="CU104" t="n">
+        <v>0.0117706684572229</v>
+      </c>
+      <c r="CV104" t="n">
+        <v>0.000433819062604638</v>
+      </c>
+      <c r="CW104" t="n">
+        <v>-0.0105359108288862</v>
+      </c>
+      <c r="CX104" t="n">
+        <v>-0.0166541341125448</v>
+      </c>
+      <c r="CY104" t="n">
+        <v>-0.0255097214412567</v>
+      </c>
+      <c r="CZ104" t="n">
+        <v>-0.0339685603302476</v>
+      </c>
+      <c r="DA104" t="n">
+        <v>-0.042361543124324</v>
+      </c>
+      <c r="DB104" t="n">
+        <v>0.0144743383069812</v>
+      </c>
+      <c r="DC104" t="n">
+        <v>0.00663991154296846</v>
+      </c>
+      <c r="DD104" t="n">
+        <v>-0.00417469876846925</v>
+      </c>
+      <c r="DE104" t="n">
+        <v>-0.0116006898326333</v>
+      </c>
+      <c r="DF104" t="n">
+        <v>-0.0259891167207186</v>
+      </c>
+      <c r="DG104" t="n">
+        <v>-0.0427394007332192</v>
+      </c>
+      <c r="DH104" t="n">
+        <v>-0.0621003069365241</v>
+      </c>
+      <c r="DI104" t="n">
+        <v>-0.123480070160362</v>
+      </c>
+      <c r="DJ104" t="n">
+        <v>-0.00235987389556172</v>
+      </c>
+      <c r="DK104" t="n">
+        <v>0.0710783358746803</v>
+      </c>
+      <c r="DL104" t="n">
+        <v>0.0637377123583466</v>
+      </c>
+      <c r="DM104" t="n">
+        <v>0.0463654743824763</v>
+      </c>
+      <c r="DN104" t="n">
+        <v>-0.00862522311551581</v>
+      </c>
+      <c r="DO104" t="n">
+        <v>-0.101035525767867</v>
+      </c>
+      <c r="DP104" t="n">
+        <v>-0.00258405583626517</v>
+      </c>
+      <c r="DQ104" t="n">
+        <v>-0.00963858878606657</v>
+      </c>
+      <c r="DR104" t="n">
+        <v>-0.0136772829791202</v>
+      </c>
+      <c r="DS104" t="n">
+        <v>-0.0163206354134338</v>
+      </c>
+      <c r="DT104" t="n">
+        <v>-0.0147366452693482</v>
+      </c>
+      <c r="DU104" t="n">
+        <v>-0.0105368446218372</v>
+      </c>
+      <c r="DV104" t="n">
+        <v>-0.00403654036919093</v>
+      </c>
+      <c r="DW104" t="n">
+        <v>0.0710227886853477</v>
+      </c>
+      <c r="DX104" t="n">
+        <v>-0.0139082060570903</v>
+      </c>
+      <c r="DY104" t="n">
+        <v>-0.0651262406312859</v>
+      </c>
+      <c r="DZ104" t="n">
+        <v>-0.0650381355054301</v>
+      </c>
+      <c r="EA104" t="n">
+        <v>-0.0522166615613574</v>
+      </c>
+      <c r="EB104" t="n">
+        <v>-0.0124070532924332</v>
+      </c>
+      <c r="EC104" t="n">
+        <v>0.0537359590573702</v>
+      </c>
+      <c r="ED104" t="n">
+        <v>0.0635423764011865</v>
+      </c>
+      <c r="EE104" t="n">
+        <v>-0.0165375345556607</v>
+      </c>
+      <c r="EF104" t="n">
+        <v>-0.0649307389190361</v>
+      </c>
+      <c r="EG104" t="n">
+        <v>-0.0662202232309161</v>
+      </c>
+      <c r="EH104" t="n">
+        <v>-0.0543932332768772</v>
+      </c>
+      <c r="EI104" t="n">
+        <v>-0.0171120190848718</v>
+      </c>
+      <c r="EJ104" t="n">
+        <v>0.0448928014068914</v>
+      </c>
+      <c r="EK104" t="n">
+        <v>0.0460910889433103</v>
+      </c>
+      <c r="EL104" t="n">
+        <v>-0.014793445074836</v>
+      </c>
+      <c r="EM104" t="n">
+        <v>-0.0518441423128612</v>
+      </c>
+      <c r="EN104" t="n">
+        <v>-0.0540537347531441</v>
+      </c>
+      <c r="EO104" t="n">
+        <v>-0.0457442159646021</v>
+      </c>
+      <c r="EP104" t="n">
+        <v>-0.0182176429715886</v>
+      </c>
+      <c r="EQ104" t="n">
+        <v>0.0278673185969962</v>
+      </c>
+      <c r="ER104" t="n">
+        <v>-0.00843403296093921</v>
+      </c>
+      <c r="ES104" t="n">
+        <v>-0.010478570685216</v>
+      </c>
+      <c r="ET104" t="n">
+        <v>-0.0123169961304431</v>
+      </c>
+      <c r="EU104" t="n">
+        <v>-0.0169352501277208</v>
+      </c>
+      <c r="EV104" t="n">
+        <v>-0.0182230972737331</v>
+      </c>
+      <c r="EW104" t="n">
+        <v>-0.019072655413115</v>
+      </c>
+      <c r="EX104" t="n">
+        <v>-0.0198771121371542</v>
+      </c>
+      <c r="EY104" t="n">
+        <v>-0.100431852799952</v>
+      </c>
+      <c r="EZ104" t="n">
+        <v>-0.00396508231012921</v>
+      </c>
+      <c r="FA104" t="n">
+        <v>0.0532882928529297</v>
+      </c>
+      <c r="FB104" t="n">
+        <v>0.0446268799495408</v>
+      </c>
+      <c r="FC104" t="n">
+        <v>0.0276273223285841</v>
+      </c>
+      <c r="FD104" t="n">
+        <v>-0.0202277299030339</v>
+      </c>
+      <c r="FE104" t="n">
+        <v>-0.0989295270162497</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -48867,6 +50667,366 @@
       <c r="AO105" t="n">
         <v>-0.0159486479837035</v>
       </c>
+      <c r="AP105" t="n">
+        <v>-0.105146210305563</v>
+      </c>
+      <c r="AQ105" t="n">
+        <v>-0.0692857420490577</v>
+      </c>
+      <c r="AR105" t="n">
+        <v>0.00511217720514391</v>
+      </c>
+      <c r="AS105" t="n">
+        <v>0.0459684613461803</v>
+      </c>
+      <c r="AT105" t="n">
+        <v>0.0368907920091629</v>
+      </c>
+      <c r="AU105" t="n">
+        <v>0.0160288265628845</v>
+      </c>
+      <c r="AV105" t="n">
+        <v>-0.032083145420225</v>
+      </c>
+      <c r="AW105" t="n">
+        <v>-0.106559864023892</v>
+      </c>
+      <c r="AX105" t="n">
+        <v>0.0317506083771615</v>
+      </c>
+      <c r="AY105" t="n">
+        <v>0.0113502966272127</v>
+      </c>
+      <c r="AZ105" t="n">
+        <v>-0.00859475936038336</v>
+      </c>
+      <c r="BA105" t="n">
+        <v>-0.0161852439823108</v>
+      </c>
+      <c r="BB105" t="n">
+        <v>-0.0324279390825786</v>
+      </c>
+      <c r="BC105" t="n">
+        <v>-0.0483006640213994</v>
+      </c>
+      <c r="BD105" t="n">
+        <v>-0.064674983623854</v>
+      </c>
+      <c r="BE105" t="n">
+        <v>0.185585132164572</v>
+      </c>
+      <c r="BF105" t="n">
+        <v>0.0137163698047325</v>
+      </c>
+      <c r="BG105" t="n">
+        <v>-0.100921466606249</v>
+      </c>
+      <c r="BH105" t="n">
+        <v>-0.104924777479181</v>
+      </c>
+      <c r="BI105" t="n">
+        <v>-0.107702394750123</v>
+      </c>
+      <c r="BJ105" t="n">
+        <v>-0.0640539431244757</v>
+      </c>
+      <c r="BK105" t="n">
+        <v>0.0225241868173211</v>
+      </c>
+      <c r="BL105" t="n">
+        <v>-0.0481666556458225</v>
+      </c>
+      <c r="BM105" t="n">
+        <v>-0.0232810207282942</v>
+      </c>
+      <c r="BN105" t="n">
+        <v>-0.00286235722617469</v>
+      </c>
+      <c r="BO105" t="n">
+        <v>-0.00426618330818394</v>
+      </c>
+      <c r="BP105" t="n">
+        <v>0.00530586561822015</v>
+      </c>
+      <c r="BQ105" t="n">
+        <v>0.0110056494363749</v>
+      </c>
+      <c r="BR105" t="n">
+        <v>0.013549068853592</v>
+      </c>
+      <c r="BS105" t="n">
+        <v>-0.0232617193305679</v>
+      </c>
+      <c r="BT105" t="n">
+        <v>-0.0166508708117211</v>
+      </c>
+      <c r="BU105" t="n">
+        <v>-0.0097645790592553</v>
+      </c>
+      <c r="BV105" t="n">
+        <v>-0.0118301557379247</v>
+      </c>
+      <c r="BW105" t="n">
+        <v>-0.00583469074098154</v>
+      </c>
+      <c r="BX105" t="n">
+        <v>0.000188985662246162</v>
+      </c>
+      <c r="BY105" t="n">
+        <v>0.00649598430673722</v>
+      </c>
+      <c r="BZ105" t="n">
+        <v>-0.00285156592227368</v>
+      </c>
+      <c r="CA105" t="n">
+        <v>-0.00989904160516603</v>
+      </c>
+      <c r="CB105" t="n">
+        <v>-0.0137683798693991</v>
+      </c>
+      <c r="CC105" t="n">
+        <v>-0.016722214126231</v>
+      </c>
+      <c r="CD105" t="n">
+        <v>-0.0149870646019586</v>
+      </c>
+      <c r="CE105" t="n">
+        <v>-0.0108114132801255</v>
+      </c>
+      <c r="CF105" t="n">
+        <v>-0.00432636030013206</v>
+      </c>
+      <c r="CG105" t="n">
+        <v>-0.00389379755579671</v>
+      </c>
+      <c r="CH105" t="n">
+        <v>-0.0117161536648343</v>
+      </c>
+      <c r="CI105" t="n">
+        <v>-0.0164299797226116</v>
+      </c>
+      <c r="CJ105" t="n">
+        <v>-0.0207339167145939</v>
+      </c>
+      <c r="CK105" t="n">
+        <v>-0.0198932260178807</v>
+      </c>
+      <c r="CL105" t="n">
+        <v>-0.0167130249750953</v>
+      </c>
+      <c r="CM105" t="n">
+        <v>-0.011356809149272</v>
+      </c>
+      <c r="CN105" t="n">
+        <v>0.0050797381506595</v>
+      </c>
+      <c r="CO105" t="n">
+        <v>-0.0061704565335063</v>
+      </c>
+      <c r="CP105" t="n">
+        <v>-0.0149191311924654</v>
+      </c>
+      <c r="CQ105" t="n">
+        <v>-0.0202312634986375</v>
+      </c>
+      <c r="CR105" t="n">
+        <v>-0.0237890779773134</v>
+      </c>
+      <c r="CS105" t="n">
+        <v>-0.0254603561989372</v>
+      </c>
+      <c r="CT105" t="n">
+        <v>-0.0256138682911627</v>
+      </c>
+      <c r="CU105" t="n">
+        <v>0.0113613627371851</v>
+      </c>
+      <c r="CV105" t="n">
+        <v>0.000118609469233599</v>
+      </c>
+      <c r="CW105" t="n">
+        <v>-0.0106718734745448</v>
+      </c>
+      <c r="CX105" t="n">
+        <v>-0.0169984806003801</v>
+      </c>
+      <c r="CY105" t="n">
+        <v>-0.0256021024779568</v>
+      </c>
+      <c r="CZ105" t="n">
+        <v>-0.0339354071858584</v>
+      </c>
+      <c r="DA105" t="n">
+        <v>-0.0424863647168434</v>
+      </c>
+      <c r="DB105" t="n">
+        <v>0.0136910216563365</v>
+      </c>
+      <c r="DC105" t="n">
+        <v>0.00632678011553616</v>
+      </c>
+      <c r="DD105" t="n">
+        <v>-0.00409729491466676</v>
+      </c>
+      <c r="DE105" t="n">
+        <v>-0.0115522115296692</v>
+      </c>
+      <c r="DF105" t="n">
+        <v>-0.0255719538540932</v>
+      </c>
+      <c r="DG105" t="n">
+        <v>-0.0421214916085836</v>
+      </c>
+      <c r="DH105" t="n">
+        <v>-0.0617499948149867</v>
+      </c>
+      <c r="DI105" t="n">
+        <v>-0.124473245859639</v>
+      </c>
+      <c r="DJ105" t="n">
+        <v>-0.00336834998990768</v>
+      </c>
+      <c r="DK105" t="n">
+        <v>0.0701438116953408</v>
+      </c>
+      <c r="DL105" t="n">
+        <v>0.0628464519743103</v>
+      </c>
+      <c r="DM105" t="n">
+        <v>0.0464464311914645</v>
+      </c>
+      <c r="DN105" t="n">
+        <v>-0.00863722202372176</v>
+      </c>
+      <c r="DO105" t="n">
+        <v>-0.100475750273934</v>
+      </c>
+      <c r="DP105" t="n">
+        <v>-0.0029011516689783</v>
+      </c>
+      <c r="DQ105" t="n">
+        <v>-0.0100240807791031</v>
+      </c>
+      <c r="DR105" t="n">
+        <v>-0.0138777530914756</v>
+      </c>
+      <c r="DS105" t="n">
+        <v>-0.0167742890162611</v>
+      </c>
+      <c r="DT105" t="n">
+        <v>-0.0148822241063267</v>
+      </c>
+      <c r="DU105" t="n">
+        <v>-0.010483376931534</v>
+      </c>
+      <c r="DV105" t="n">
+        <v>-0.00369836523569771</v>
+      </c>
+      <c r="DW105" t="n">
+        <v>0.0706055318996815</v>
+      </c>
+      <c r="DX105" t="n">
+        <v>-0.0138268103651276</v>
+      </c>
+      <c r="DY105" t="n">
+        <v>-0.0644554288752727</v>
+      </c>
+      <c r="DZ105" t="n">
+        <v>-0.064843306294611</v>
+      </c>
+      <c r="EA105" t="n">
+        <v>-0.052244791471519</v>
+      </c>
+      <c r="EB105" t="n">
+        <v>-0.0124096871542396</v>
+      </c>
+      <c r="EC105" t="n">
+        <v>0.0532958538082202</v>
+      </c>
+      <c r="ED105" t="n">
+        <v>0.0641441128885326</v>
+      </c>
+      <c r="EE105" t="n">
+        <v>-0.0165074018855961</v>
+      </c>
+      <c r="EF105" t="n">
+        <v>-0.064896361898445</v>
+      </c>
+      <c r="EG105" t="n">
+        <v>-0.0666507345010892</v>
+      </c>
+      <c r="EH105" t="n">
+        <v>-0.0547698292436291</v>
+      </c>
+      <c r="EI105" t="n">
+        <v>-0.0169476346959692</v>
+      </c>
+      <c r="EJ105" t="n">
+        <v>0.0454940121045415</v>
+      </c>
+      <c r="EK105" t="n">
+        <v>0.0461739325363401</v>
+      </c>
+      <c r="EL105" t="n">
+        <v>-0.0149089295565116</v>
+      </c>
+      <c r="EM105" t="n">
+        <v>-0.0517940075556908</v>
+      </c>
+      <c r="EN105" t="n">
+        <v>-0.0545113506481571</v>
+      </c>
+      <c r="EO105" t="n">
+        <v>-0.0461847586418263</v>
+      </c>
+      <c r="EP105" t="n">
+        <v>-0.0184450907593058</v>
+      </c>
+      <c r="EQ105" t="n">
+        <v>0.0276727077061971</v>
+      </c>
+      <c r="ER105" t="n">
+        <v>-0.00852562546952068</v>
+      </c>
+      <c r="ES105" t="n">
+        <v>-0.0105950795275189</v>
+      </c>
+      <c r="ET105" t="n">
+        <v>-0.0122882249320182</v>
+      </c>
+      <c r="EU105" t="n">
+        <v>-0.0172463293023774</v>
+      </c>
+      <c r="EV105" t="n">
+        <v>-0.018363329761079</v>
+      </c>
+      <c r="EW105" t="n">
+        <v>-0.0193494654482249</v>
+      </c>
+      <c r="EX105" t="n">
+        <v>-0.0203299367906181</v>
+      </c>
+      <c r="EY105" t="n">
+        <v>-0.101251812249911</v>
+      </c>
+      <c r="EZ105" t="n">
+        <v>-0.00399047032100493</v>
+      </c>
+      <c r="FA105" t="n">
+        <v>0.0537382047518536</v>
+      </c>
+      <c r="FB105" t="n">
+        <v>0.0450783861806746</v>
+      </c>
+      <c r="FC105" t="n">
+        <v>0.0285385522062384</v>
+      </c>
+      <c r="FD105" t="n">
+        <v>-0.0201847253467146</v>
+      </c>
+      <c r="FE105" t="n">
+        <v>-0.0996482627601939</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -48991,6 +51151,366 @@
       </c>
       <c r="AO106" t="n">
         <v>-0.0165147169474905</v>
+      </c>
+      <c r="AP106" t="n">
+        <v>-0.105550553663153</v>
+      </c>
+      <c r="AQ106" t="n">
+        <v>-0.0688495393506358</v>
+      </c>
+      <c r="AR106" t="n">
+        <v>0.00554278258900663</v>
+      </c>
+      <c r="AS106" t="n">
+        <v>0.0463802955063233</v>
+      </c>
+      <c r="AT106" t="n">
+        <v>0.0368607084881188</v>
+      </c>
+      <c r="AU106" t="n">
+        <v>0.0157839685626136</v>
+      </c>
+      <c r="AV106" t="n">
+        <v>-0.0323240781745767</v>
+      </c>
+      <c r="AW106" t="n">
+        <v>-0.107214509560368</v>
+      </c>
+      <c r="AX106" t="n">
+        <v>0.0321909582294015</v>
+      </c>
+      <c r="AY106" t="n">
+        <v>0.0111339198202389</v>
+      </c>
+      <c r="AZ106" t="n">
+        <v>-0.00898904139180593</v>
+      </c>
+      <c r="BA106" t="n">
+        <v>-0.0166888948700315</v>
+      </c>
+      <c r="BB106" t="n">
+        <v>-0.0325331752057351</v>
+      </c>
+      <c r="BC106" t="n">
+        <v>-0.0485700751691266</v>
+      </c>
+      <c r="BD106" t="n">
+        <v>-0.0641438678431801</v>
+      </c>
+      <c r="BE106" t="n">
+        <v>0.184466026560489</v>
+      </c>
+      <c r="BF106" t="n">
+        <v>0.0128024780765051</v>
+      </c>
+      <c r="BG106" t="n">
+        <v>-0.101230006978942</v>
+      </c>
+      <c r="BH106" t="n">
+        <v>-0.10480478310846</v>
+      </c>
+      <c r="BI106" t="n">
+        <v>-0.106761159947139</v>
+      </c>
+      <c r="BJ106" t="n">
+        <v>-0.0645900618397775</v>
+      </c>
+      <c r="BK106" t="n">
+        <v>0.0228945764614509</v>
+      </c>
+      <c r="BL106" t="n">
+        <v>-0.0469187894799061</v>
+      </c>
+      <c r="BM106" t="n">
+        <v>-0.0227837345279208</v>
+      </c>
+      <c r="BN106" t="n">
+        <v>-0.00291750796947706</v>
+      </c>
+      <c r="BO106" t="n">
+        <v>-0.00392829880599033</v>
+      </c>
+      <c r="BP106" t="n">
+        <v>0.00539279230079919</v>
+      </c>
+      <c r="BQ106" t="n">
+        <v>0.0115529952711843</v>
+      </c>
+      <c r="BR106" t="n">
+        <v>0.0143654107211105</v>
+      </c>
+      <c r="BS106" t="n">
+        <v>-0.0228041342935668</v>
+      </c>
+      <c r="BT106" t="n">
+        <v>-0.0165812622720381</v>
+      </c>
+      <c r="BU106" t="n">
+        <v>-0.00993527088844883</v>
+      </c>
+      <c r="BV106" t="n">
+        <v>-0.0117449933921144</v>
+      </c>
+      <c r="BW106" t="n">
+        <v>-0.00585200641871301</v>
+      </c>
+      <c r="BX106" t="n">
+        <v>0.000366779601482206</v>
+      </c>
+      <c r="BY106" t="n">
+        <v>0.00689871553572618</v>
+      </c>
+      <c r="BZ106" t="n">
+        <v>-0.00244654279466072</v>
+      </c>
+      <c r="CA106" t="n">
+        <v>-0.00983556071782374</v>
+      </c>
+      <c r="CB106" t="n">
+        <v>-0.0139105472065549</v>
+      </c>
+      <c r="CC106" t="n">
+        <v>-0.016738901829918</v>
+      </c>
+      <c r="CD106" t="n">
+        <v>-0.0151311319554657</v>
+      </c>
+      <c r="CE106" t="n">
+        <v>-0.0111390219558903</v>
+      </c>
+      <c r="CF106" t="n">
+        <v>-0.00460330560994081</v>
+      </c>
+      <c r="CG106" t="n">
+        <v>-0.00342774470450474</v>
+      </c>
+      <c r="CH106" t="n">
+        <v>-0.01163878960696</v>
+      </c>
+      <c r="CI106" t="n">
+        <v>-0.0165742831771284</v>
+      </c>
+      <c r="CJ106" t="n">
+        <v>-0.0207396908654182</v>
+      </c>
+      <c r="CK106" t="n">
+        <v>-0.0200441636435413</v>
+      </c>
+      <c r="CL106" t="n">
+        <v>-0.0171084132258173</v>
+      </c>
+      <c r="CM106" t="n">
+        <v>-0.0116960832793683</v>
+      </c>
+      <c r="CN106" t="n">
+        <v>0.00549638899580102</v>
+      </c>
+      <c r="CO106" t="n">
+        <v>-0.00600731253491179</v>
+      </c>
+      <c r="CP106" t="n">
+        <v>-0.0148289417295588</v>
+      </c>
+      <c r="CQ106" t="n">
+        <v>-0.0199732925231662</v>
+      </c>
+      <c r="CR106" t="n">
+        <v>-0.0235117828284143</v>
+      </c>
+      <c r="CS106" t="n">
+        <v>-0.0254376123881714</v>
+      </c>
+      <c r="CT106" t="n">
+        <v>-0.0253980587460751</v>
+      </c>
+      <c r="CU106" t="n">
+        <v>0.0113901961031073</v>
+      </c>
+      <c r="CV106" t="n">
+        <v>0.000115528541358177</v>
+      </c>
+      <c r="CW106" t="n">
+        <v>-0.0105298003003169</v>
+      </c>
+      <c r="CX106" t="n">
+        <v>-0.0167748797302233</v>
+      </c>
+      <c r="CY106" t="n">
+        <v>-0.0251919670608419</v>
+      </c>
+      <c r="CZ106" t="n">
+        <v>-0.0337688342549331</v>
+      </c>
+      <c r="DA106" t="n">
+        <v>-0.0420498115321095</v>
+      </c>
+      <c r="DB106" t="n">
+        <v>0.0135818664328444</v>
+      </c>
+      <c r="DC106" t="n">
+        <v>0.00619383818525349</v>
+      </c>
+      <c r="DD106" t="n">
+        <v>-0.0040152362115934</v>
+      </c>
+      <c r="DE106" t="n">
+        <v>-0.0114958546443047</v>
+      </c>
+      <c r="DF106" t="n">
+        <v>-0.025181426606578</v>
+      </c>
+      <c r="DG106" t="n">
+        <v>-0.041896828429579</v>
+      </c>
+      <c r="DH106" t="n">
+        <v>-0.0610851840259746</v>
+      </c>
+      <c r="DI106" t="n">
+        <v>-0.124147104360027</v>
+      </c>
+      <c r="DJ106" t="n">
+        <v>-0.00253157788899357</v>
+      </c>
+      <c r="DK106" t="n">
+        <v>0.0711772063303095</v>
+      </c>
+      <c r="DL106" t="n">
+        <v>0.0635156307998679</v>
+      </c>
+      <c r="DM106" t="n">
+        <v>0.0466826471323351</v>
+      </c>
+      <c r="DN106" t="n">
+        <v>-0.00802244258867711</v>
+      </c>
+      <c r="DO106" t="n">
+        <v>-0.100755563207552</v>
+      </c>
+      <c r="DP106" t="n">
+        <v>-0.00285981693482858</v>
+      </c>
+      <c r="DQ106" t="n">
+        <v>-0.00995040706604706</v>
+      </c>
+      <c r="DR106" t="n">
+        <v>-0.0137487818928308</v>
+      </c>
+      <c r="DS106" t="n">
+        <v>-0.0164696562440681</v>
+      </c>
+      <c r="DT106" t="n">
+        <v>-0.0146557195815404</v>
+      </c>
+      <c r="DU106" t="n">
+        <v>-0.0104631918309034</v>
+      </c>
+      <c r="DV106" t="n">
+        <v>-0.00373922683128239</v>
+      </c>
+      <c r="DW106" t="n">
+        <v>0.0708373273270795</v>
+      </c>
+      <c r="DX106" t="n">
+        <v>-0.0141535525546207</v>
+      </c>
+      <c r="DY106" t="n">
+        <v>-0.0649973187663387</v>
+      </c>
+      <c r="DZ106" t="n">
+        <v>-0.0648580602571258</v>
+      </c>
+      <c r="EA106" t="n">
+        <v>-0.0521014231474126</v>
+      </c>
+      <c r="EB106" t="n">
+        <v>-0.0127238118746736</v>
+      </c>
+      <c r="EC106" t="n">
+        <v>0.0536262096103437</v>
+      </c>
+      <c r="ED106" t="n">
+        <v>0.0638789479152368</v>
+      </c>
+      <c r="EE106" t="n">
+        <v>-0.016779810078942</v>
+      </c>
+      <c r="EF106" t="n">
+        <v>-0.0650434818267197</v>
+      </c>
+      <c r="EG106" t="n">
+        <v>-0.0662816225649614</v>
+      </c>
+      <c r="EH106" t="n">
+        <v>-0.0543662334734076</v>
+      </c>
+      <c r="EI106" t="n">
+        <v>-0.0172985358685832</v>
+      </c>
+      <c r="EJ106" t="n">
+        <v>0.045317731809575</v>
+      </c>
+      <c r="EK106" t="n">
+        <v>0.0467586328239622</v>
+      </c>
+      <c r="EL106" t="n">
+        <v>-0.0149394752551705</v>
+      </c>
+      <c r="EM106" t="n">
+        <v>-0.0520789955714353</v>
+      </c>
+      <c r="EN106" t="n">
+        <v>-0.0542740927640672</v>
+      </c>
+      <c r="EO106" t="n">
+        <v>-0.0458341597231142</v>
+      </c>
+      <c r="EP106" t="n">
+        <v>-0.0184310465572626</v>
+      </c>
+      <c r="EQ106" t="n">
+        <v>0.0283067216073548</v>
+      </c>
+      <c r="ER106" t="n">
+        <v>-0.00853361180353372</v>
+      </c>
+      <c r="ES106" t="n">
+        <v>-0.0104070854091085</v>
+      </c>
+      <c r="ET106" t="n">
+        <v>-0.0119189194110935</v>
+      </c>
+      <c r="EU106" t="n">
+        <v>-0.016699136368092</v>
+      </c>
+      <c r="EV106" t="n">
+        <v>-0.0179198097431885</v>
+      </c>
+      <c r="EW106" t="n">
+        <v>-0.0192391294669925</v>
+      </c>
+      <c r="EX106" t="n">
+        <v>-0.0204042132423705</v>
+      </c>
+      <c r="EY106" t="n">
+        <v>-0.100667901832558</v>
+      </c>
+      <c r="EZ106" t="n">
+        <v>-0.00352070024148432</v>
+      </c>
+      <c r="FA106" t="n">
+        <v>0.0541091935054595</v>
+      </c>
+      <c r="FB106" t="n">
+        <v>0.0451206174209094</v>
+      </c>
+      <c r="FC106" t="n">
+        <v>0.028339100267032</v>
+      </c>
+      <c r="FD106" t="n">
+        <v>-0.0199457190403841</v>
+      </c>
+      <c r="FE106" t="n">
+        <v>-0.0996849198481287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>